<commit_message>
panel de beneficios instalados
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\curso_big_data\ejercicios_excell\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D895D6-1F1E-444F-BDCC-F0864E7BBCC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D6A07E-D2CB-407E-B542-970034530BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,6 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -650,6 +648,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -684,20 +696,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -709,6 +707,580 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Dispersion</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t>: Coste vs Beneficio</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$B$5:$B$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>80</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$C$5:$C$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>15.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9CA7-40A6-9720-BB88AB83D247}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1924039951"/>
+        <c:axId val="1924038511"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1924039951"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1924038511"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1924038511"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1924039951"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
 </file>
 
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -787,6 +1359,46 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1334,6 +1946,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1417,8 +2545,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2499440-986D-CADD-6ECE-ED9880888E63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38E5041C-F245-4966-82E1-642C61AE9389}" name="Tabla1" displayName="Tabla1" ref="A1:N43" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38E5041C-F245-4966-82E1-642C61AE9389}" name="Tabla1" displayName="Tabla1" ref="A1:N43" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:N43" xr:uid="{38E5041C-F245-4966-82E1-642C61AE9389}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{CD681CD3-B8DF-41F4-B1C1-97FF537BD801}" name="ID_Venta"/>
@@ -4062,7 +5231,7 @@
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -4100,7 +5269,10 @@
       <c r="E5" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="4">
+        <f>AVERAGE(C5:C46)</f>
+        <v>32.511904761904759</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -4115,7 +5287,10 @@
       <c r="E6" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="4">
+        <f>_xlfn.STDEV.S(C5:C46)</f>
+        <v>20.550499399082351</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -4130,7 +5305,10 @@
       <c r="E7" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="4">
+        <f>MIN(C5:C46)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -4145,7 +5323,10 @@
       <c r="E8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="4">
+        <f>MAX(C5:C46)</f>
+        <v>120</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -4570,6 +5751,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Valoracion de satisfaccion terminada
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\curso_big_data\ejercicios_excell\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D6A07E-D2CB-407E-B542-970034530BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F288B8-25E8-4B0A-86EE-B6E7EA5C0CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -1283,6 +1283,381 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Distribucion de satisfaccion</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.36523600174978127"/>
+          <c:y val="5.5555555555555552E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$D$12:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$E$12:$E$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-151E-4B52-91C0-1D85D54FB56D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="529963200"/>
+        <c:axId val="529967040"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="529963200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="529967040"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="529967040"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="529963200"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1438,6 +1813,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2443,6 +2858,509 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -2566,6 +3484,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2499440-986D-CADD-6ECE-ED9880888E63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A5AD02C-A399-E87E-9825-A83C2AF9E300}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5762,7 +6721,7 @@
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="30.21875" customWidth="1"/>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5795,7 +6754,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>4.2857142857142856</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -5807,7 +6769,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -5819,7 +6784,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -5872,7 +6840,10 @@
       <c r="D12" s="3">
         <v>1</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4">
+        <f>COUNTIF($B$5:$B$46,D12)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -5884,7 +6855,10 @@
       <c r="D13" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4">
+        <f t="shared" ref="E13:E16" si="0">COUNTIF($B$5:$B$46,D13)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -5896,7 +6870,10 @@
       <c r="D14" s="3">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="4">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -5908,7 +6885,10 @@
       <c r="D15" s="3">
         <v>4</v>
       </c>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -5920,7 +6900,10 @@
       <c r="D16" s="3">
         <v>5</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -6167,6 +7150,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>